<commit_message>
Week 02 Day 02 data Cleaning succesfully implemented
</commit_message>
<xml_diff>
--- a/Month-01-Excel/Week-01/Day -05/Day-05-Excel-Workbook.xlsx
+++ b/Month-01-Excel/Week-01/Day -05/Day-05-Excel-Workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\4_MONTH\4-Month-Data-Analyst-Journey\Month-01-Excel\Week-01\Day -05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F6A65A-5D30-488E-9586-BB50A358AD49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE1EE5D6-B225-4793-A852-B139D18EDA89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tutorial" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -288,9 +288,6 @@
     <t xml:space="preserve">bussniness ques 4 </t>
   </si>
   <si>
-    <t>DAY 05 — CONDITIONAL FUNCTIONS</t>
-  </si>
-  <si>
     <t>SUMIF</t>
   </si>
   <si>
@@ -364,13 +361,16 @@
   </si>
   <si>
     <t>Verify Result</t>
+  </si>
+  <si>
+    <t>]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -457,89 +457,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFA9D08E"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFA9D08E"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -816,9 +761,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -829,7 +774,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -844,7 +789,7 @@
         <v>#NAME?</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -855,7 +800,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -866,7 +811,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
@@ -877,7 +822,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
         <v>0</v>
       </c>
@@ -888,7 +833,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
@@ -921,7 +866,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81A756FD-B80C-47C3-BABB-FB06EA6772C6}">
   <dimension ref="A1:J22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.42578125" customWidth="1"/>
@@ -931,7 +876,7 @@
     <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10">
       <c r="A1" s="4" t="s">
         <v>10</v>
       </c>
@@ -963,7 +908,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10">
       <c r="A2" s="4"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -982,7 +927,7 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10">
       <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
@@ -1009,7 +954,7 @@
         <f>COUNTIF(D3:D22,"&gt;40000")</f>
         <v>8</v>
       </c>
-      <c r="I3" s="11">
+      <c r="I3" s="9">
         <f>SUMIFS(D3:D22,B3:B22,"North",C3:C22,"Electronics")</f>
         <v>161000</v>
       </c>
@@ -1018,7 +963,7 @@
         <v>169000</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10">
       <c r="A4" s="5" t="s">
         <v>19</v>
       </c>
@@ -1043,7 +988,7 @@
       <c r="H4" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="9">
         <f>SUMIFS(D3:D22,B3:B22,"North",C3:C22,"Furniture")</f>
         <v>61000</v>
       </c>
@@ -1052,7 +997,7 @@
         <v>172000</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10">
       <c r="A5" s="5" t="s">
         <v>22</v>
       </c>
@@ -1071,7 +1016,7 @@
       <c r="F5" s="5">
         <v>2</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="9">
         <f>SUM(D:D)</f>
         <v>713000</v>
       </c>
@@ -1088,7 +1033,7 @@
         <v>128000</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10">
       <c r="A6" s="5" t="s">
         <v>23</v>
       </c>
@@ -1118,7 +1063,7 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10">
       <c r="A7" s="5" t="s">
         <v>25</v>
       </c>
@@ -1137,11 +1082,11 @@
       <c r="F7" s="5">
         <v>5</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="9">
         <f>SUMIF(B:B,B4,D:D)</f>
         <v>169000</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="9">
         <f>SUMIF(D3:D22,"&gt;40000",E3:E22)</f>
         <v>74000</v>
       </c>
@@ -1152,7 +1097,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10">
       <c r="A8" s="5" t="s">
         <v>28</v>
       </c>
@@ -1174,7 +1119,7 @@
       <c r="G8" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="12" t="s">
         <v>57</v>
       </c>
       <c r="I8" s="7">
@@ -1186,7 +1131,7 @@
         <v>116000</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10">
       <c r="A9" s="5" t="s">
         <v>29</v>
       </c>
@@ -1205,11 +1150,11 @@
       <c r="F9" s="5">
         <v>2</v>
       </c>
-      <c r="G9" s="11">
+      <c r="G9" s="9">
         <f>COUNTIF(B:B,"North")</f>
         <v>6</v>
       </c>
-      <c r="H9" s="15">
+      <c r="H9" s="13">
         <f>AVERAGEIF(D3:D22,"&gt;=3",F3:F22)</f>
         <v>3.15</v>
       </c>
@@ -1218,7 +1163,7 @@
         <v>5857.1428571428569</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10">
       <c r="A10" s="5" t="s">
         <v>30</v>
       </c>
@@ -1240,13 +1185,12 @@
       <c r="G10" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="H10" s="13"/>
       <c r="I10" s="3">
         <f>AVERAGEIF(C3:C22,"Clothing",E3:E22)</f>
         <v>3940</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10">
       <c r="A11" s="5" t="s">
         <v>31</v>
       </c>
@@ -1265,13 +1209,12 @@
       <c r="F11" s="5">
         <v>3</v>
       </c>
-      <c r="G11" s="11">
+      <c r="G11" s="9">
         <f>COUNTIF(C:C,C5)</f>
         <v>7</v>
       </c>
-      <c r="H11" s="13"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:10">
       <c r="A12" s="5" t="s">
         <v>32</v>
       </c>
@@ -1293,9 +1236,8 @@
       <c r="G12" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="H12" s="13"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:10">
       <c r="A13" s="5" t="s">
         <v>33</v>
       </c>
@@ -1314,13 +1256,12 @@
       <c r="F13" s="5">
         <v>3</v>
       </c>
-      <c r="G13" s="11">
+      <c r="G13" s="9">
         <f>SUMIFS(D3:D22,B3:B22,"North",C3:C22,"Furniture")</f>
         <v>61000</v>
       </c>
-      <c r="H13" s="13"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:10">
       <c r="A14" s="5" t="s">
         <v>34</v>
       </c>
@@ -1342,10 +1283,8 @@
       <c r="G14" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:10">
       <c r="A15" s="5" t="s">
         <v>35</v>
       </c>
@@ -1364,13 +1303,12 @@
       <c r="F15" s="5">
         <v>2</v>
       </c>
-      <c r="G15" s="11">
+      <c r="G15" s="9">
         <f>SUMIFS(E3:E22,B3:B22,"South",C3:C22,"Electronics")</f>
         <v>15000</v>
       </c>
-      <c r="H15" s="13"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:10">
       <c r="A16" s="5" t="s">
         <v>36</v>
       </c>
@@ -1392,9 +1330,8 @@
       <c r="G16" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="H16" s="13"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:7">
       <c r="A17" s="5" t="s">
         <v>37</v>
       </c>
@@ -1413,13 +1350,12 @@
       <c r="F17" s="5">
         <v>5</v>
       </c>
-      <c r="G17" s="12">
+      <c r="G17" s="11">
         <f>AVERAGEIF(B3:B22,"North",D3:D22)</f>
         <v>40666.666666666664</v>
       </c>
-      <c r="H17" s="13"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18" s="5" t="s">
         <v>38</v>
       </c>
@@ -1441,9 +1377,8 @@
       <c r="G18" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="H18" s="13"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:7">
       <c r="A19" s="5" t="s">
         <v>39</v>
       </c>
@@ -1462,13 +1397,12 @@
       <c r="F19" s="5">
         <v>4</v>
       </c>
-      <c r="G19" s="11">
+      <c r="G19" s="9">
         <f>AVERAGEIF(C3:C22,"Electronics",E3:E22)</f>
         <v>9187.5</v>
       </c>
-      <c r="H19" s="13"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:7">
       <c r="A20" s="5" t="s">
         <v>40</v>
       </c>
@@ -1490,9 +1424,8 @@
       <c r="G20" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="H20" s="13"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
         <v>41</v>
       </c>
@@ -1511,13 +1444,12 @@
       <c r="F21" s="5">
         <v>3</v>
       </c>
-      <c r="G21" s="12">
+      <c r="G21" s="11">
         <f>AVERAGEIFS(D3:D22,B3:B22,"North",C3:C22,"Electronics")</f>
         <v>53666.666666666664</v>
       </c>
-      <c r="H21" s="13"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22" s="5" t="s">
         <v>42</v>
       </c>
@@ -1536,8 +1468,7 @@
       <c r="F22" s="5">
         <v>2</v>
       </c>
-      <c r="G22" s="11"/>
-      <c r="H22" s="13"/>
+      <c r="G22" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1547,156 +1478,156 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4864B474-B507-4F9E-A47D-6E2B7BA65031}">
   <dimension ref="A1:A40"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="12" spans="1:1">
+      <c r="A12" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="13" spans="1:1">
+      <c r="A13" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="15" spans="1:1">
+      <c r="A15" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="16" spans="1:1">
+      <c r="A16" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="21" spans="1:1">
+      <c r="A21" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="26" spans="1:1">
+      <c r="A26" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="28" spans="1:1">
+      <c r="A28" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="29" spans="1:1">
+      <c r="A29" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="31" spans="1:1">
+      <c r="A31" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1">
       <c r="A32" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1">
       <c r="A33" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="35" spans="1:1">
+      <c r="A35" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="37" spans="1:1">
+      <c r="A37" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="39" spans="1:1">
+      <c r="A39" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>